<commit_message>
Site guncellemesi - 24.09.2026 18:51
</commit_message>
<xml_diff>
--- a/app/borsa/gosterge-taramalari/data/rsi40-alti.xlsx
+++ b/app/borsa/gosterge-taramalari/data/rsi40-alti.xlsx
@@ -53,6 +53,9 @@
     <x:t>AFYON</x:t>
   </x:si>
   <x:si>
+    <x:t>AGESA</x:t>
+  </x:si>
+  <x:si>
     <x:t>AGROT</x:t>
   </x:si>
   <x:si>
@@ -65,6 +68,9 @@
     <x:t>AKENR</x:t>
   </x:si>
   <x:si>
+    <x:t>AKFYE</x:t>
+  </x:si>
+  <x:si>
     <x:t>AKGRT</x:t>
   </x:si>
   <x:si>
@@ -125,6 +131,9 @@
     <x:t>ARASE</x:t>
   </x:si>
   <x:si>
+    <x:t>ARCLK</x:t>
+  </x:si>
+  <x:si>
     <x:t>ARDYZ</x:t>
   </x:si>
   <x:si>
@@ -146,6 +155,9 @@
     <x:t>ASGYO</x:t>
   </x:si>
   <x:si>
+    <x:t>ASTOR</x:t>
+  </x:si>
+  <x:si>
     <x:t>ASUZU</x:t>
   </x:si>
   <x:si>
@@ -155,6 +167,9 @@
     <x:t>ATAKP</x:t>
   </x:si>
   <x:si>
+    <x:t>ATATP</x:t>
+  </x:si>
+  <x:si>
     <x:t>ATATR</x:t>
   </x:si>
   <x:si>
@@ -176,12 +191,18 @@
     <x:t>AYCES</x:t>
   </x:si>
   <x:si>
+    <x:t>AYDEM</x:t>
+  </x:si>
+  <x:si>
     <x:t>AYEN</x:t>
   </x:si>
   <x:si>
     <x:t>AYES</x:t>
   </x:si>
   <x:si>
+    <x:t>AZTEK</x:t>
+  </x:si>
+  <x:si>
     <x:t>BAGFS</x:t>
   </x:si>
   <x:si>
@@ -215,6 +236,9 @@
     <x:t>BERA</x:t>
   </x:si>
   <x:si>
+    <x:t>BESLR</x:t>
+  </x:si>
+  <x:si>
     <x:t>BESTE</x:t>
   </x:si>
   <x:si>
@@ -254,1521 +278,1518 @@
     <x:t>BJKAS</x:t>
   </x:si>
   <x:si>
+    <x:t>BMSCH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BNTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BOBET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BORLS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BORSK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRISA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRKSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRKVY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRLSM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRMEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRYAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BSOKE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BTCIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BUCIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BULGS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BURCE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BURVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BVSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BYDNR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CANTE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CASA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CATES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CEMAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CEMTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CEMZY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CEOEM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CGCAM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CLEBI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CMBTN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CMENT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CONSE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>COSMO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CRDFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CUSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CWENE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DAGI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DAPGM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DARDL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DCTTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DENGE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DERHL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DERIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DESA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DESPC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DGATE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DGGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DGNMO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DIRIT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DITAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DMRGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DMSAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DNISI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOCO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOFER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOFRB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOGUB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOKTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DSTKF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DUNYH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DURKN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DYOBY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DZGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ECOGR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ECZYT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EDATA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EDIP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EFOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGEGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGEPO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGSER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKDMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKIZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKSUN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ELITE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMKEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMPAE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENDAE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENPRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENSRI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ERBOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ERCB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ERSU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ESCAR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ESCOM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ESEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ETYAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUKYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUPWR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUREN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EUYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EYGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FADE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FENER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FONET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FORMT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FORTE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FRIGO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FRMPL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FZLGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GARFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GATEG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEDIK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEDZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GENIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GENKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GENTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GEREL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GESAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GIPTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLCVY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLRMK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLRYH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOKNR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOLDA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOLTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOODY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GOZDE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GRNYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GRSEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GRTHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GSDDE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GSDHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GSRAY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUNDG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GWIND</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GZNMI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HATEK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HATSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HDFGS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HEDEF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HEKTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HKTM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HLGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HOROZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HTTBT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUBVC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HURGZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ICBCT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ICUGS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IDGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IEYHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHAAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHEVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHGZT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHLAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHLGM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IHYAY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IMASM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INDES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INFO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INGRM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INTEK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INTEM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INVEO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>INVES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISBIR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISBTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISFIN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISGSY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISKPL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISSEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISVEA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IZENR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IZFAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IZINV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IZMDC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JANTS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAPLM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KARCL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAREL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KARSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KARTN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KATMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAYSE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KBORU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KCAER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KENT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KFEIN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KIMMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLKIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLMSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLNMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLRHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLSER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLYPV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KMPUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KNFRT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOCMT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KONKA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KONTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOPOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KORDS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KOTON</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KPEKS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRDMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRDMB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRSTL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KSTUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KTLEV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KTSKR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KUTPO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KUVVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KUYAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KZBGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KZGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LIDER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LILAK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LINK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LKMNH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LRSHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LUKSK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LXGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LYDHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LYDYE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAALT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MACKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAGEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAKIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAKTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MANAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARBL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARTI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MCARD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEDTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEGAP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEGMT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEKAG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MERCN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MERIT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MERKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>METRO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEYSU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MHRGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MIATK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MMCAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MNDRS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MNDTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MOBTL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MOGAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MOPAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MRGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MSGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MTRKS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MZHLD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NATEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NETCD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NIBAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NTGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NTHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NUGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OBAMS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OBASE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ODINE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ONCSM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ONRYT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORCAY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORZAX</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OSMEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OSTIM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OTTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OYAYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OYLUM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OYYAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZATD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZKGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OZRDN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAMEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PAPIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PARSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PASEU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PATEK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PEKGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PENGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PENTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PINSU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PKART</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PKENT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PLTUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PNLSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>POLHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>POLTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRDGS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRKAB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRKME</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PRZMA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PSDTC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PSGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QNBFK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QNBTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QUAGR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QUICK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RALYH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RAYSG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>REEDR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RNPOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RODRG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RTALB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RUBNS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RUZYE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAFKR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAMAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SANEL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SANFM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SANKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SARAE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SARKY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SASA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SAYAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SDTTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEGMN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEKFK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEKUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SELEC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SELVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SERNT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SEYKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SILVR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKBNK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SKYLP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SMART</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SMRTG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SMRVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SNGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SNICA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SODSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SOHOE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SOKE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SONME</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SRVGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SSAAT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SUMAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SUNTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SURGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SUWEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SVGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TABGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TARKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TATEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TCKRC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TDGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TEHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TEKTU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TERA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TEZOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TGSAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TKNKA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TKNSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TLMAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TMPOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TMSN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TRILC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TSGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TSKB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TSPOR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TURGG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UCAYM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>UFUK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULUFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULUSE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ULUUN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>USAK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKFN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VAKKO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VANGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VBTYZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VERTU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VERUS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VESBE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VESTL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VEYAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VKFYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VKGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VKING</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VRGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>VSNMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YAPRK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YATAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YAYLA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YBTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YEOTK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YESIL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YGGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YIGIT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YKSLN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YONGA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YUNSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YYAPI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YYLGD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ZEDUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ZERGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ZGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ZOREN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ADGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AEFES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AGHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AHGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKBNK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKCNS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKFGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKFIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AKSGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALARK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALBRK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANHYT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ASELS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ATEKS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AVGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AVPGY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AYGAZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BAHKM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BIMAS</x:t>
+  </x:si>
+  <x:si>
     <x:t>BLCYT</x:t>
   </x:si>
   <x:si>
-    <x:t>BMSCH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BNTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BOBET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BORLS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BORSK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRKSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRKVY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRLSM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRMEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRYAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BSOKE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BTCIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BUCIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BULGS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BURCE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BURVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BVSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BYDNR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CASA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CATES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CEMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CEMTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CEMZY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CGCAM</x:t>
+    <x:t>BLUME</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BMSTL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BOSSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>BRSAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CCOLA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CELHA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>CIMSA</x:t>
   </x:si>
   <x:si>
     <x:t>CITAS</x:t>
   </x:si>
   <x:si>
-    <x:t>CMENT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CONSE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>COSMO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CRDFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CUSAN</x:t>
+    <x:t>CRFSA</x:t>
   </x:si>
   <x:si>
     <x:t>CVKMD</x:t>
   </x:si>
   <x:si>
-    <x:t>CWENE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DAGI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DAPGM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DARDL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DCTTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DENGE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DERHL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DERIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DESA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DESPC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DGATE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DGGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DGNMO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DIRIT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DITAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DMRGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DMSAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DNISI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOCO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOFER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOFRB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOGUB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOKTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DSTKF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DUNYH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURKN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DYOBY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ECOGR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ECZYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EDATA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EDIP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EFOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGEGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGEPO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGSER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKIZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKSUN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ELITE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMKEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMPAE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENDAE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENPRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENSRI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ERBOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ERCB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ERSU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ESCAR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ESCOM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ESEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETYAT</x:t>
+    <x:t>DEVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DURDO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EBEBK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ECILC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGEEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGGUB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EGPRO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EKGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMNIS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENERY</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENJSA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENKAI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ENTRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EPLAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EREGL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ETILR</x:t>
   </x:si>
   <x:si>
     <x:t>EUHOL</x:t>
   </x:si>
   <x:si>
-    <x:t>EUKYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUPWR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUREN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EUYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EYGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FADE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FENER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FONET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FORMT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FORTE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FRIGO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FRMPL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FZLGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GARFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GATEG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEDIK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEDZA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GENIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GENKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GENTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GEREL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GESAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GIPTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLCVY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLRMK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLRYH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOKNR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOLDA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOLTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOODY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GOZDE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GRNYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GRSEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GRTHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GSDHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GSRAY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUNDG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GWIND</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GZNMI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HATEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HATSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HDFGS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HEDEF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HEKTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HKTM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HOROZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HTTBT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUBVC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HURGZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ICBCT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ICUGS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IDGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IEYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHAAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHGZT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHLAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHLGM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IHYAY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IMASM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INFO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INGRM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INTEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INTEM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INVEO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISBIR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISBTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISGSY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISKPL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISSEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISVEA</x:t>
+    <x:t>FLAP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FMIZP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FROTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GARAN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLBMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GLYHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GMTAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUBRF</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HALKB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HRKET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HUNER</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISATR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISCTR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISDMR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISGYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISKUR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISMEN</x:t>
   </x:si>
   <x:si>
     <x:t>ISYAT</x:t>
   </x:si>
   <x:si>
-    <x:t>IZENR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IZFAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IZINV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IZMDC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAPLM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAREL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KARTN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KATMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAYSE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KBORU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KCAER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KENT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KFEIN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KIMMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLKIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLMSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLNMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLRHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLSER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLYPV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KMPUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KOCMT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KONKA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KONTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KOPOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KORDS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KOTON</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KPEKS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMB</x:t>
+    <x:t>KCHOL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KERVN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KLSYN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KONYA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRDMD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRGYO</x:t>
   </x:si>
   <x:si>
     <x:t>KRONT</x:t>
   </x:si>
   <x:si>
-    <x:t>KRSTL</x:t>
+    <x:t>KRPLS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KRTEK</x:t>
   </x:si>
   <x:si>
     <x:t>KRVGD</x:t>
   </x:si>
   <x:si>
-    <x:t>KSTUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KTLEV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KTSKR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KUTPO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KUVVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KUYAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KZBGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KZGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LIDER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LILAK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LINK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LKMNH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LRSHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LUKSK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LXGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LYDHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LYDYE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAALT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MACKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAGEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAKIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAKTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MANAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARBL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARTI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MCARD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEDTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEGAP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEGMT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEKAG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MERCN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MERIT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MERKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>METRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEYSU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MHRGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MIATK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MMCAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MNDRS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MNDTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MOBTL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MOGAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MOPAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MRGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MSGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MTRKS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MZHLD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NATEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NETCD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NIBAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NTHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NUGYO</x:t>
+    <x:t>LIDFA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LMKDC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LOGO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MASFN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MAVI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MEPET</x:t>
+  </x:si>
+  <x:si>
+    <x:t>METEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MGROS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MPARK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MRSHL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MTRYO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NETAS</x:t>
   </x:si>
   <x:si>
     <x:t>NUHCM</x:t>
   </x:si>
   <x:si>
-    <x:t>OBAMS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OBASE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ODINE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ONCSM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ONRYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORCAY</x:t>
+    <x:t>ODAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OFSYM</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ORGE</x:t>
   </x:si>
   <x:si>
     <x:t>ORMA</x:t>
   </x:si>
   <x:si>
-    <x:t>ORZAX</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OSMEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OSTIM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OTTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OYAYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OYLUM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OYYAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZATD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OZRDN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAMEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAPIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PARSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PASEU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PATEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PEKGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PENGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PENTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PINSU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PKART</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PKENT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PLTUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PNLSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>POLHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>POLTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRDGS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRKAB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRKME</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PRZMA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PSDTC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PSGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QNBFK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QNBTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QUAGR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>QUICK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RALYH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RAYSG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>REEDR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RNPOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RODRG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RTALB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RUBNS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RUZYE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SAFKR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SAMAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SANEL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SANFM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SARAE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SARKY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SASA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SAYAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SDTTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEGMN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEKFK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEKUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SELEC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SELVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SERNT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SEYKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SILVR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKBNK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SKYLP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SMART</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SMRTG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SMRVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SNGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SNICA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SODSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOHOE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SOKE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SONME</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SRVGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SSAAT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SUMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SUNTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SURGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SUWEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SVGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TABGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TARKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TATEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TDGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TEHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TEKTU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TERA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TEZOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TGSAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKNKA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TKNSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TLMAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TMPOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TMSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TRILC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TSGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TSPOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UCAYM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UFUK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULUFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULUSE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ULUUN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>USAK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKFN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VAKKO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VANGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VBTYZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VERTU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VERUS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VESBE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VEYAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VKFYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VKGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VKING</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VRGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VSNMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YAPRK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YATAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YAYLA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YBTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YESIL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YIGIT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YKSLN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YONGA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YUNSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YYAPI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YYLGD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ZEDUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ZERGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ZGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ZOREN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ADGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AEFES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AGESA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AGHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AHGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKBNK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKCNS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKFGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKFIS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKFYE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AKSGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALARK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALBRK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANHYT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARCLK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ARSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ASELS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ASTOR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATATP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ATEKS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AVPGY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYDEM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AYGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AZTEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BAHKM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BESLR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BIMAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BLUME</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BMSTL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BOSSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRISA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BRSAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CANTE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CCOLA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CELHA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CEOEM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CIMSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CLEBI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CMBTN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>CRFSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DEVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DURDO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DZGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EBEBK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ECILC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGEEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGGUB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EGPRO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EKGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMNIS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENERY</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENJSA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENKAI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ENTRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EPLAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EREGL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ETILR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FLAP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FMIZP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FROTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GARAN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLBMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GLYHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GMTAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GSDDE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUBRF</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HALKB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HLGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HRKET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HUNER</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INDES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>INVES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISATR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISCTR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISDMR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISFIN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISKUR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISMEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JANTS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KARCL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KARSN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KCHOL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KERVN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KLSYN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KNFRT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KONYA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRDMD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRGYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRPLS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KRTEK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LIDFA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LMKDC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LOGO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MASFN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MAVI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MEPET</x:t>
-  </x:si>
-  <x:si>
-    <x:t>METEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MGROS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MPARK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MRSHL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MTRYO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NETAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NTGAZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ODAS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OFSYM</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ORGE</x:t>
-  </x:si>
-  <x:si>
     <x:t>OTKAR</x:t>
   </x:si>
   <x:si>
     <x:t>OYAKC</x:t>
   </x:si>
   <x:si>
-    <x:t>OZKGY</x:t>
-  </x:si>
-  <x:si>
     <x:t>OZSUB</x:t>
   </x:si>
   <x:si>
@@ -1802,9 +1823,6 @@
     <x:t>SAHOL</x:t>
   </x:si>
   <x:si>
-    <x:t>SANKO</x:t>
-  </x:si>
-  <x:si>
     <x:t>SISE</x:t>
   </x:si>
   <x:si>
@@ -1829,9 +1847,6 @@
     <x:t>TCELL</x:t>
   </x:si>
   <x:si>
-    <x:t>TCKRC</x:t>
-  </x:si>
-  <x:si>
     <x:t>THYAO</x:t>
   </x:si>
   <x:si>
@@ -1859,9 +1874,6 @@
     <x:t>TRMET</x:t>
   </x:si>
   <x:si>
-    <x:t>TSKB</x:t>
-  </x:si>
-  <x:si>
     <x:t>TTKOM</x:t>
   </x:si>
   <x:si>
@@ -1880,9 +1892,6 @@
     <x:t>TUREX</x:t>
   </x:si>
   <x:si>
-    <x:t>TURGG</x:t>
-  </x:si>
-  <x:si>
     <x:t>TURSG</x:t>
   </x:si>
   <x:si>
@@ -1896,15 +1905,6 @@
   </x:si>
   <x:si>
     <x:t>VAKBN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>VESTL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YEOTK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YGGYO</x:t>
   </x:si>
   <x:si>
     <x:t>YKBNK</x:t>
@@ -2261,7 +2261,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C467"/>
+  <x:dimension ref="A1:C491"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -7398,6 +7398,270 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C467" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="468" spans="1:3">
+      <x:c r="A468" s="0" t="s">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="B468" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C468" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="469" spans="1:3">
+      <x:c r="A469" s="0" t="s">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="B469" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C469" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="470" spans="1:3">
+      <x:c r="A470" s="0" t="s">
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="B470" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C470" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="471" spans="1:3">
+      <x:c r="A471" s="0" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="B471" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C471" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="472" spans="1:3">
+      <x:c r="A472" s="0" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="B472" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C472" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="473" spans="1:3">
+      <x:c r="A473" s="0" t="s">
+        <x:v>476</x:v>
+      </x:c>
+      <x:c r="B473" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C473" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="474" spans="1:3">
+      <x:c r="A474" s="0" t="s">
+        <x:v>477</x:v>
+      </x:c>
+      <x:c r="B474" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C474" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="475" spans="1:3">
+      <x:c r="A475" s="0" t="s">
+        <x:v>478</x:v>
+      </x:c>
+      <x:c r="B475" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C475" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="476" spans="1:3">
+      <x:c r="A476" s="0" t="s">
+        <x:v>479</x:v>
+      </x:c>
+      <x:c r="B476" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C476" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="477" spans="1:3">
+      <x:c r="A477" s="0" t="s">
+        <x:v>480</x:v>
+      </x:c>
+      <x:c r="B477" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C477" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="478" spans="1:3">
+      <x:c r="A478" s="0" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="B478" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C478" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="479" spans="1:3">
+      <x:c r="A479" s="0" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="B479" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C479" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="480" spans="1:3">
+      <x:c r="A480" s="0" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="B480" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C480" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="481" spans="1:3">
+      <x:c r="A481" s="0" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="B481" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C481" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="482" spans="1:3">
+      <x:c r="A482" s="0" t="s">
+        <x:v>485</x:v>
+      </x:c>
+      <x:c r="B482" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C482" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="483" spans="1:3">
+      <x:c r="A483" s="0" t="s">
+        <x:v>486</x:v>
+      </x:c>
+      <x:c r="B483" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C483" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="484" spans="1:3">
+      <x:c r="A484" s="0" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="B484" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C484" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="485" spans="1:3">
+      <x:c r="A485" s="0" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="B485" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C485" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="486" spans="1:3">
+      <x:c r="A486" s="0" t="s">
+        <x:v>489</x:v>
+      </x:c>
+      <x:c r="B486" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C486" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="487" spans="1:3">
+      <x:c r="A487" s="0" t="s">
+        <x:v>490</x:v>
+      </x:c>
+      <x:c r="B487" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C487" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="488" spans="1:3">
+      <x:c r="A488" s="0" t="s">
+        <x:v>491</x:v>
+      </x:c>
+      <x:c r="B488" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C488" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="489" spans="1:3">
+      <x:c r="A489" s="0" t="s">
+        <x:v>492</x:v>
+      </x:c>
+      <x:c r="B489" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C489" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="490" spans="1:3">
+      <x:c r="A490" s="0" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="B490" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C490" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="491" spans="1:3">
+      <x:c r="A491" s="0" t="s">
+        <x:v>494</x:v>
+      </x:c>
+      <x:c r="B491" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C491" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -7415,7 +7679,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:C162"/>
+  <x:dimension ref="A1:C138"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:3">
@@ -7431,7 +7695,7 @@
     </x:row>
     <x:row r="2" spans="1:3">
       <x:c r="A2" s="0" t="s">
-        <x:v>471</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
         <x:v>4</x:v>
@@ -7442,7 +7706,7 @@
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="0" t="s">
-        <x:v>472</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
         <x:v>4</x:v>
@@ -7453,7 +7717,7 @@
     </x:row>
     <x:row r="4" spans="1:3">
       <x:c r="A4" s="0" t="s">
-        <x:v>473</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
         <x:v>4</x:v>
@@ -7464,7 +7728,7 @@
     </x:row>
     <x:row r="5" spans="1:3">
       <x:c r="A5" s="0" t="s">
-        <x:v>474</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
         <x:v>4</x:v>
@@ -7475,7 +7739,7 @@
     </x:row>
     <x:row r="6" spans="1:3">
       <x:c r="A6" s="0" t="s">
-        <x:v>475</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>4</x:v>
@@ -7486,7 +7750,7 @@
     </x:row>
     <x:row r="7" spans="1:3">
       <x:c r="A7" s="0" t="s">
-        <x:v>476</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>4</x:v>
@@ -7497,7 +7761,7 @@
     </x:row>
     <x:row r="8" spans="1:3">
       <x:c r="A8" s="0" t="s">
-        <x:v>477</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>4</x:v>
@@ -7508,7 +7772,7 @@
     </x:row>
     <x:row r="9" spans="1:3">
       <x:c r="A9" s="0" t="s">
-        <x:v>478</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>4</x:v>
@@ -7519,7 +7783,7 @@
     </x:row>
     <x:row r="10" spans="1:3">
       <x:c r="A10" s="0" t="s">
-        <x:v>479</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
         <x:v>4</x:v>
@@ -7530,7 +7794,7 @@
     </x:row>
     <x:row r="11" spans="1:3">
       <x:c r="A11" s="0" t="s">
-        <x:v>480</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
         <x:v>4</x:v>
@@ -7541,7 +7805,7 @@
     </x:row>
     <x:row r="12" spans="1:3">
       <x:c r="A12" s="0" t="s">
-        <x:v>481</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
         <x:v>4</x:v>
@@ -7552,7 +7816,7 @@
     </x:row>
     <x:row r="13" spans="1:3">
       <x:c r="A13" s="0" t="s">
-        <x:v>482</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
         <x:v>4</x:v>
@@ -7563,7 +7827,7 @@
     </x:row>
     <x:row r="14" spans="1:3">
       <x:c r="A14" s="0" t="s">
-        <x:v>483</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
         <x:v>4</x:v>
@@ -7574,7 +7838,7 @@
     </x:row>
     <x:row r="15" spans="1:3">
       <x:c r="A15" s="0" t="s">
-        <x:v>484</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
         <x:v>4</x:v>
@@ -7585,7 +7849,7 @@
     </x:row>
     <x:row r="16" spans="1:3">
       <x:c r="A16" s="0" t="s">
-        <x:v>485</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
         <x:v>4</x:v>
@@ -7596,7 +7860,7 @@
     </x:row>
     <x:row r="17" spans="1:3">
       <x:c r="A17" s="0" t="s">
-        <x:v>486</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
         <x:v>4</x:v>
@@ -7607,7 +7871,7 @@
     </x:row>
     <x:row r="18" spans="1:3">
       <x:c r="A18" s="0" t="s">
-        <x:v>487</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
         <x:v>4</x:v>
@@ -7618,7 +7882,7 @@
     </x:row>
     <x:row r="19" spans="1:3">
       <x:c r="A19" s="0" t="s">
-        <x:v>488</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
         <x:v>4</x:v>
@@ -7629,7 +7893,7 @@
     </x:row>
     <x:row r="20" spans="1:3">
       <x:c r="A20" s="0" t="s">
-        <x:v>489</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
         <x:v>4</x:v>
@@ -7640,7 +7904,7 @@
     </x:row>
     <x:row r="21" spans="1:3">
       <x:c r="A21" s="0" t="s">
-        <x:v>490</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
         <x:v>4</x:v>
@@ -7651,7 +7915,7 @@
     </x:row>
     <x:row r="22" spans="1:3">
       <x:c r="A22" s="0" t="s">
-        <x:v>491</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
         <x:v>4</x:v>
@@ -7662,7 +7926,7 @@
     </x:row>
     <x:row r="23" spans="1:3">
       <x:c r="A23" s="0" t="s">
-        <x:v>492</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
         <x:v>4</x:v>
@@ -7673,7 +7937,7 @@
     </x:row>
     <x:row r="24" spans="1:3">
       <x:c r="A24" s="0" t="s">
-        <x:v>493</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
         <x:v>4</x:v>
@@ -7684,7 +7948,7 @@
     </x:row>
     <x:row r="25" spans="1:3">
       <x:c r="A25" s="0" t="s">
-        <x:v>494</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
         <x:v>4</x:v>
@@ -7695,7 +7959,7 @@
     </x:row>
     <x:row r="26" spans="1:3">
       <x:c r="A26" s="0" t="s">
-        <x:v>495</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
         <x:v>4</x:v>
@@ -7706,7 +7970,7 @@
     </x:row>
     <x:row r="27" spans="1:3">
       <x:c r="A27" s="0" t="s">
-        <x:v>496</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
         <x:v>4</x:v>
@@ -7717,7 +7981,7 @@
     </x:row>
     <x:row r="28" spans="1:3">
       <x:c r="A28" s="0" t="s">
-        <x:v>497</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
         <x:v>4</x:v>
@@ -7728,7 +7992,7 @@
     </x:row>
     <x:row r="29" spans="1:3">
       <x:c r="A29" s="0" t="s">
-        <x:v>498</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
         <x:v>4</x:v>
@@ -7739,7 +8003,7 @@
     </x:row>
     <x:row r="30" spans="1:3">
       <x:c r="A30" s="0" t="s">
-        <x:v>499</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
         <x:v>4</x:v>
@@ -7750,7 +8014,7 @@
     </x:row>
     <x:row r="31" spans="1:3">
       <x:c r="A31" s="0" t="s">
-        <x:v>500</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
         <x:v>4</x:v>
@@ -7761,7 +8025,7 @@
     </x:row>
     <x:row r="32" spans="1:3">
       <x:c r="A32" s="0" t="s">
-        <x:v>501</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
         <x:v>4</x:v>
@@ -7772,7 +8036,7 @@
     </x:row>
     <x:row r="33" spans="1:3">
       <x:c r="A33" s="0" t="s">
-        <x:v>502</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
         <x:v>4</x:v>
@@ -7783,7 +8047,7 @@
     </x:row>
     <x:row r="34" spans="1:3">
       <x:c r="A34" s="0" t="s">
-        <x:v>503</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
         <x:v>4</x:v>
@@ -7794,7 +8058,7 @@
     </x:row>
     <x:row r="35" spans="1:3">
       <x:c r="A35" s="0" t="s">
-        <x:v>504</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
         <x:v>4</x:v>
@@ -7805,7 +8069,7 @@
     </x:row>
     <x:row r="36" spans="1:3">
       <x:c r="A36" s="0" t="s">
-        <x:v>505</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
         <x:v>4</x:v>
@@ -7816,7 +8080,7 @@
     </x:row>
     <x:row r="37" spans="1:3">
       <x:c r="A37" s="0" t="s">
-        <x:v>506</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
         <x:v>4</x:v>
@@ -7827,7 +8091,7 @@
     </x:row>
     <x:row r="38" spans="1:3">
       <x:c r="A38" s="0" t="s">
-        <x:v>507</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
         <x:v>4</x:v>
@@ -7838,7 +8102,7 @@
     </x:row>
     <x:row r="39" spans="1:3">
       <x:c r="A39" s="0" t="s">
-        <x:v>508</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
         <x:v>4</x:v>
@@ -7849,7 +8113,7 @@
     </x:row>
     <x:row r="40" spans="1:3">
       <x:c r="A40" s="0" t="s">
-        <x:v>509</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
         <x:v>4</x:v>
@@ -7860,7 +8124,7 @@
     </x:row>
     <x:row r="41" spans="1:3">
       <x:c r="A41" s="0" t="s">
-        <x:v>510</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="B41" s="0" t="s">
         <x:v>4</x:v>
@@ -7871,7 +8135,7 @@
     </x:row>
     <x:row r="42" spans="1:3">
       <x:c r="A42" s="0" t="s">
-        <x:v>511</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="B42" s="0" t="s">
         <x:v>4</x:v>
@@ -7882,7 +8146,7 @@
     </x:row>
     <x:row r="43" spans="1:3">
       <x:c r="A43" s="0" t="s">
-        <x:v>512</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="B43" s="0" t="s">
         <x:v>4</x:v>
@@ -7893,7 +8157,7 @@
     </x:row>
     <x:row r="44" spans="1:3">
       <x:c r="A44" s="0" t="s">
-        <x:v>513</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="B44" s="0" t="s">
         <x:v>4</x:v>
@@ -7904,7 +8168,7 @@
     </x:row>
     <x:row r="45" spans="1:3">
       <x:c r="A45" s="0" t="s">
-        <x:v>514</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="B45" s="0" t="s">
         <x:v>4</x:v>
@@ -7915,7 +8179,7 @@
     </x:row>
     <x:row r="46" spans="1:3">
       <x:c r="A46" s="0" t="s">
-        <x:v>515</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="B46" s="0" t="s">
         <x:v>4</x:v>
@@ -7926,7 +8190,7 @@
     </x:row>
     <x:row r="47" spans="1:3">
       <x:c r="A47" s="0" t="s">
-        <x:v>516</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="B47" s="0" t="s">
         <x:v>4</x:v>
@@ -7937,7 +8201,7 @@
     </x:row>
     <x:row r="48" spans="1:3">
       <x:c r="A48" s="0" t="s">
-        <x:v>517</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="B48" s="0" t="s">
         <x:v>4</x:v>
@@ -7948,7 +8212,7 @@
     </x:row>
     <x:row r="49" spans="1:3">
       <x:c r="A49" s="0" t="s">
-        <x:v>518</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B49" s="0" t="s">
         <x:v>4</x:v>
@@ -7959,7 +8223,7 @@
     </x:row>
     <x:row r="50" spans="1:3">
       <x:c r="A50" s="0" t="s">
-        <x:v>519</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="B50" s="0" t="s">
         <x:v>4</x:v>
@@ -7970,7 +8234,7 @@
     </x:row>
     <x:row r="51" spans="1:3">
       <x:c r="A51" s="0" t="s">
-        <x:v>520</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="B51" s="0" t="s">
         <x:v>4</x:v>
@@ -7981,7 +8245,7 @@
     </x:row>
     <x:row r="52" spans="1:3">
       <x:c r="A52" s="0" t="s">
-        <x:v>521</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="B52" s="0" t="s">
         <x:v>4</x:v>
@@ -7992,7 +8256,7 @@
     </x:row>
     <x:row r="53" spans="1:3">
       <x:c r="A53" s="0" t="s">
-        <x:v>522</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="B53" s="0" t="s">
         <x:v>4</x:v>
@@ -8003,7 +8267,7 @@
     </x:row>
     <x:row r="54" spans="1:3">
       <x:c r="A54" s="0" t="s">
-        <x:v>523</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="B54" s="0" t="s">
         <x:v>4</x:v>
@@ -8014,7 +8278,7 @@
     </x:row>
     <x:row r="55" spans="1:3">
       <x:c r="A55" s="0" t="s">
-        <x:v>524</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="B55" s="0" t="s">
         <x:v>4</x:v>
@@ -8025,7 +8289,7 @@
     </x:row>
     <x:row r="56" spans="1:3">
       <x:c r="A56" s="0" t="s">
-        <x:v>525</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="B56" s="0" t="s">
         <x:v>4</x:v>
@@ -8036,7 +8300,7 @@
     </x:row>
     <x:row r="57" spans="1:3">
       <x:c r="A57" s="0" t="s">
-        <x:v>526</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="B57" s="0" t="s">
         <x:v>4</x:v>
@@ -8047,7 +8311,7 @@
     </x:row>
     <x:row r="58" spans="1:3">
       <x:c r="A58" s="0" t="s">
-        <x:v>527</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="B58" s="0" t="s">
         <x:v>4</x:v>
@@ -8058,7 +8322,7 @@
     </x:row>
     <x:row r="59" spans="1:3">
       <x:c r="A59" s="0" t="s">
-        <x:v>528</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="B59" s="0" t="s">
         <x:v>4</x:v>
@@ -8069,7 +8333,7 @@
     </x:row>
     <x:row r="60" spans="1:3">
       <x:c r="A60" s="0" t="s">
-        <x:v>529</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="B60" s="0" t="s">
         <x:v>4</x:v>
@@ -8080,7 +8344,7 @@
     </x:row>
     <x:row r="61" spans="1:3">
       <x:c r="A61" s="0" t="s">
-        <x:v>530</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="B61" s="0" t="s">
         <x:v>4</x:v>
@@ -8091,7 +8355,7 @@
     </x:row>
     <x:row r="62" spans="1:3">
       <x:c r="A62" s="0" t="s">
-        <x:v>531</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="B62" s="0" t="s">
         <x:v>4</x:v>
@@ -8102,7 +8366,7 @@
     </x:row>
     <x:row r="63" spans="1:3">
       <x:c r="A63" s="0" t="s">
-        <x:v>532</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="B63" s="0" t="s">
         <x:v>4</x:v>
@@ -8113,7 +8377,7 @@
     </x:row>
     <x:row r="64" spans="1:3">
       <x:c r="A64" s="0" t="s">
-        <x:v>533</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="B64" s="0" t="s">
         <x:v>4</x:v>
@@ -8124,7 +8388,7 @@
     </x:row>
     <x:row r="65" spans="1:3">
       <x:c r="A65" s="0" t="s">
-        <x:v>534</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="B65" s="0" t="s">
         <x:v>4</x:v>
@@ -8135,7 +8399,7 @@
     </x:row>
     <x:row r="66" spans="1:3">
       <x:c r="A66" s="0" t="s">
-        <x:v>535</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="B66" s="0" t="s">
         <x:v>4</x:v>
@@ -8146,7 +8410,7 @@
     </x:row>
     <x:row r="67" spans="1:3">
       <x:c r="A67" s="0" t="s">
-        <x:v>536</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="B67" s="0" t="s">
         <x:v>4</x:v>
@@ -8157,7 +8421,7 @@
     </x:row>
     <x:row r="68" spans="1:3">
       <x:c r="A68" s="0" t="s">
-        <x:v>537</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="B68" s="0" t="s">
         <x:v>4</x:v>
@@ -8168,7 +8432,7 @@
     </x:row>
     <x:row r="69" spans="1:3">
       <x:c r="A69" s="0" t="s">
-        <x:v>538</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="B69" s="0" t="s">
         <x:v>4</x:v>
@@ -8179,7 +8443,7 @@
     </x:row>
     <x:row r="70" spans="1:3">
       <x:c r="A70" s="0" t="s">
-        <x:v>539</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="B70" s="0" t="s">
         <x:v>4</x:v>
@@ -8190,7 +8454,7 @@
     </x:row>
     <x:row r="71" spans="1:3">
       <x:c r="A71" s="0" t="s">
-        <x:v>540</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="B71" s="0" t="s">
         <x:v>4</x:v>
@@ -8201,7 +8465,7 @@
     </x:row>
     <x:row r="72" spans="1:3">
       <x:c r="A72" s="0" t="s">
-        <x:v>541</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="B72" s="0" t="s">
         <x:v>4</x:v>
@@ -8212,7 +8476,7 @@
     </x:row>
     <x:row r="73" spans="1:3">
       <x:c r="A73" s="0" t="s">
-        <x:v>542</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="B73" s="0" t="s">
         <x:v>4</x:v>
@@ -8223,7 +8487,7 @@
     </x:row>
     <x:row r="74" spans="1:3">
       <x:c r="A74" s="0" t="s">
-        <x:v>543</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B74" s="0" t="s">
         <x:v>4</x:v>
@@ -8234,7 +8498,7 @@
     </x:row>
     <x:row r="75" spans="1:3">
       <x:c r="A75" s="0" t="s">
-        <x:v>544</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="B75" s="0" t="s">
         <x:v>4</x:v>
@@ -8245,7 +8509,7 @@
     </x:row>
     <x:row r="76" spans="1:3">
       <x:c r="A76" s="0" t="s">
-        <x:v>545</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="B76" s="0" t="s">
         <x:v>4</x:v>
@@ -8256,7 +8520,7 @@
     </x:row>
     <x:row r="77" spans="1:3">
       <x:c r="A77" s="0" t="s">
-        <x:v>546</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="B77" s="0" t="s">
         <x:v>4</x:v>
@@ -8267,7 +8531,7 @@
     </x:row>
     <x:row r="78" spans="1:3">
       <x:c r="A78" s="0" t="s">
-        <x:v>547</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="B78" s="0" t="s">
         <x:v>4</x:v>
@@ -8278,7 +8542,7 @@
     </x:row>
     <x:row r="79" spans="1:3">
       <x:c r="A79" s="0" t="s">
-        <x:v>548</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="B79" s="0" t="s">
         <x:v>4</x:v>
@@ -8289,7 +8553,7 @@
     </x:row>
     <x:row r="80" spans="1:3">
       <x:c r="A80" s="0" t="s">
-        <x:v>549</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="B80" s="0" t="s">
         <x:v>4</x:v>
@@ -8300,7 +8564,7 @@
     </x:row>
     <x:row r="81" spans="1:3">
       <x:c r="A81" s="0" t="s">
-        <x:v>550</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="B81" s="0" t="s">
         <x:v>4</x:v>
@@ -8311,7 +8575,7 @@
     </x:row>
     <x:row r="82" spans="1:3">
       <x:c r="A82" s="0" t="s">
-        <x:v>551</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="B82" s="0" t="s">
         <x:v>4</x:v>
@@ -8322,7 +8586,7 @@
     </x:row>
     <x:row r="83" spans="1:3">
       <x:c r="A83" s="0" t="s">
-        <x:v>552</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="B83" s="0" t="s">
         <x:v>4</x:v>
@@ -8333,7 +8597,7 @@
     </x:row>
     <x:row r="84" spans="1:3">
       <x:c r="A84" s="0" t="s">
-        <x:v>553</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="B84" s="0" t="s">
         <x:v>4</x:v>
@@ -8344,7 +8608,7 @@
     </x:row>
     <x:row r="85" spans="1:3">
       <x:c r="A85" s="0" t="s">
-        <x:v>554</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="B85" s="0" t="s">
         <x:v>4</x:v>
@@ -8355,7 +8619,7 @@
     </x:row>
     <x:row r="86" spans="1:3">
       <x:c r="A86" s="0" t="s">
-        <x:v>555</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="B86" s="0" t="s">
         <x:v>4</x:v>
@@ -8366,7 +8630,7 @@
     </x:row>
     <x:row r="87" spans="1:3">
       <x:c r="A87" s="0" t="s">
-        <x:v>556</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="B87" s="0" t="s">
         <x:v>4</x:v>
@@ -8377,7 +8641,7 @@
     </x:row>
     <x:row r="88" spans="1:3">
       <x:c r="A88" s="0" t="s">
-        <x:v>557</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="B88" s="0" t="s">
         <x:v>4</x:v>
@@ -8388,7 +8652,7 @@
     </x:row>
     <x:row r="89" spans="1:3">
       <x:c r="A89" s="0" t="s">
-        <x:v>558</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="B89" s="0" t="s">
         <x:v>4</x:v>
@@ -8399,7 +8663,7 @@
     </x:row>
     <x:row r="90" spans="1:3">
       <x:c r="A90" s="0" t="s">
-        <x:v>559</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="B90" s="0" t="s">
         <x:v>4</x:v>
@@ -8410,7 +8674,7 @@
     </x:row>
     <x:row r="91" spans="1:3">
       <x:c r="A91" s="0" t="s">
-        <x:v>560</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="B91" s="0" t="s">
         <x:v>4</x:v>
@@ -8421,7 +8685,7 @@
     </x:row>
     <x:row r="92" spans="1:3">
       <x:c r="A92" s="0" t="s">
-        <x:v>561</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="B92" s="0" t="s">
         <x:v>4</x:v>
@@ -8432,7 +8696,7 @@
     </x:row>
     <x:row r="93" spans="1:3">
       <x:c r="A93" s="0" t="s">
-        <x:v>562</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="B93" s="0" t="s">
         <x:v>4</x:v>
@@ -8443,7 +8707,7 @@
     </x:row>
     <x:row r="94" spans="1:3">
       <x:c r="A94" s="0" t="s">
-        <x:v>563</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="B94" s="0" t="s">
         <x:v>4</x:v>
@@ -8454,7 +8718,7 @@
     </x:row>
     <x:row r="95" spans="1:3">
       <x:c r="A95" s="0" t="s">
-        <x:v>564</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="B95" s="0" t="s">
         <x:v>4</x:v>
@@ -8465,7 +8729,7 @@
     </x:row>
     <x:row r="96" spans="1:3">
       <x:c r="A96" s="0" t="s">
-        <x:v>565</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="B96" s="0" t="s">
         <x:v>4</x:v>
@@ -8476,7 +8740,7 @@
     </x:row>
     <x:row r="97" spans="1:3">
       <x:c r="A97" s="0" t="s">
-        <x:v>566</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="B97" s="0" t="s">
         <x:v>4</x:v>
@@ -8487,7 +8751,7 @@
     </x:row>
     <x:row r="98" spans="1:3">
       <x:c r="A98" s="0" t="s">
-        <x:v>567</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="B98" s="0" t="s">
         <x:v>4</x:v>
@@ -8498,7 +8762,7 @@
     </x:row>
     <x:row r="99" spans="1:3">
       <x:c r="A99" s="0" t="s">
-        <x:v>568</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="B99" s="0" t="s">
         <x:v>4</x:v>
@@ -8509,7 +8773,7 @@
     </x:row>
     <x:row r="100" spans="1:3">
       <x:c r="A100" s="0" t="s">
-        <x:v>569</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="B100" s="0" t="s">
         <x:v>4</x:v>
@@ -8520,7 +8784,7 @@
     </x:row>
     <x:row r="101" spans="1:3">
       <x:c r="A101" s="0" t="s">
-        <x:v>570</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="B101" s="0" t="s">
         <x:v>4</x:v>
@@ -8531,7 +8795,7 @@
     </x:row>
     <x:row r="102" spans="1:3">
       <x:c r="A102" s="0" t="s">
-        <x:v>571</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="B102" s="0" t="s">
         <x:v>4</x:v>
@@ -8542,7 +8806,7 @@
     </x:row>
     <x:row r="103" spans="1:3">
       <x:c r="A103" s="0" t="s">
-        <x:v>572</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="B103" s="0" t="s">
         <x:v>4</x:v>
@@ -8553,7 +8817,7 @@
     </x:row>
     <x:row r="104" spans="1:3">
       <x:c r="A104" s="0" t="s">
-        <x:v>573</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="B104" s="0" t="s">
         <x:v>4</x:v>
@@ -8564,7 +8828,7 @@
     </x:row>
     <x:row r="105" spans="1:3">
       <x:c r="A105" s="0" t="s">
-        <x:v>574</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="B105" s="0" t="s">
         <x:v>4</x:v>
@@ -8575,7 +8839,7 @@
     </x:row>
     <x:row r="106" spans="1:3">
       <x:c r="A106" s="0" t="s">
-        <x:v>575</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="B106" s="0" t="s">
         <x:v>4</x:v>
@@ -8586,7 +8850,7 @@
     </x:row>
     <x:row r="107" spans="1:3">
       <x:c r="A107" s="0" t="s">
-        <x:v>576</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="B107" s="0" t="s">
         <x:v>4</x:v>
@@ -8597,7 +8861,7 @@
     </x:row>
     <x:row r="108" spans="1:3">
       <x:c r="A108" s="0" t="s">
-        <x:v>577</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="B108" s="0" t="s">
         <x:v>4</x:v>
@@ -8608,7 +8872,7 @@
     </x:row>
     <x:row r="109" spans="1:3">
       <x:c r="A109" s="0" t="s">
-        <x:v>578</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="B109" s="0" t="s">
         <x:v>4</x:v>
@@ -8619,7 +8883,7 @@
     </x:row>
     <x:row r="110" spans="1:3">
       <x:c r="A110" s="0" t="s">
-        <x:v>579</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="B110" s="0" t="s">
         <x:v>4</x:v>
@@ -8630,7 +8894,7 @@
     </x:row>
     <x:row r="111" spans="1:3">
       <x:c r="A111" s="0" t="s">
-        <x:v>580</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="B111" s="0" t="s">
         <x:v>4</x:v>
@@ -8641,7 +8905,7 @@
     </x:row>
     <x:row r="112" spans="1:3">
       <x:c r="A112" s="0" t="s">
-        <x:v>581</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="B112" s="0" t="s">
         <x:v>4</x:v>
@@ -8652,7 +8916,7 @@
     </x:row>
     <x:row r="113" spans="1:3">
       <x:c r="A113" s="0" t="s">
-        <x:v>582</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="B113" s="0" t="s">
         <x:v>4</x:v>
@@ -8663,7 +8927,7 @@
     </x:row>
     <x:row r="114" spans="1:3">
       <x:c r="A114" s="0" t="s">
-        <x:v>583</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="B114" s="0" t="s">
         <x:v>4</x:v>
@@ -8674,7 +8938,7 @@
     </x:row>
     <x:row r="115" spans="1:3">
       <x:c r="A115" s="0" t="s">
-        <x:v>584</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="B115" s="0" t="s">
         <x:v>4</x:v>
@@ -8685,7 +8949,7 @@
     </x:row>
     <x:row r="116" spans="1:3">
       <x:c r="A116" s="0" t="s">
-        <x:v>585</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="B116" s="0" t="s">
         <x:v>4</x:v>
@@ -8696,7 +8960,7 @@
     </x:row>
     <x:row r="117" spans="1:3">
       <x:c r="A117" s="0" t="s">
-        <x:v>586</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="B117" s="0" t="s">
         <x:v>4</x:v>
@@ -8707,7 +8971,7 @@
     </x:row>
     <x:row r="118" spans="1:3">
       <x:c r="A118" s="0" t="s">
-        <x:v>587</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="B118" s="0" t="s">
         <x:v>4</x:v>
@@ -8718,7 +8982,7 @@
     </x:row>
     <x:row r="119" spans="1:3">
       <x:c r="A119" s="0" t="s">
-        <x:v>588</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="B119" s="0" t="s">
         <x:v>4</x:v>
@@ -8729,7 +8993,7 @@
     </x:row>
     <x:row r="120" spans="1:3">
       <x:c r="A120" s="0" t="s">
-        <x:v>589</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="B120" s="0" t="s">
         <x:v>4</x:v>
@@ -8740,7 +9004,7 @@
     </x:row>
     <x:row r="121" spans="1:3">
       <x:c r="A121" s="0" t="s">
-        <x:v>590</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="B121" s="0" t="s">
         <x:v>4</x:v>
@@ -8751,7 +9015,7 @@
     </x:row>
     <x:row r="122" spans="1:3">
       <x:c r="A122" s="0" t="s">
-        <x:v>591</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="B122" s="0" t="s">
         <x:v>4</x:v>
@@ -8762,7 +9026,7 @@
     </x:row>
     <x:row r="123" spans="1:3">
       <x:c r="A123" s="0" t="s">
-        <x:v>592</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="B123" s="0" t="s">
         <x:v>4</x:v>
@@ -8773,7 +9037,7 @@
     </x:row>
     <x:row r="124" spans="1:3">
       <x:c r="A124" s="0" t="s">
-        <x:v>593</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="B124" s="0" t="s">
         <x:v>4</x:v>
@@ -8784,7 +9048,7 @@
     </x:row>
     <x:row r="125" spans="1:3">
       <x:c r="A125" s="0" t="s">
-        <x:v>594</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="B125" s="0" t="s">
         <x:v>4</x:v>
@@ -8795,7 +9059,7 @@
     </x:row>
     <x:row r="126" spans="1:3">
       <x:c r="A126" s="0" t="s">
-        <x:v>595</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="B126" s="0" t="s">
         <x:v>4</x:v>
@@ -8806,7 +9070,7 @@
     </x:row>
     <x:row r="127" spans="1:3">
       <x:c r="A127" s="0" t="s">
-        <x:v>596</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="B127" s="0" t="s">
         <x:v>4</x:v>
@@ -8817,7 +9081,7 @@
     </x:row>
     <x:row r="128" spans="1:3">
       <x:c r="A128" s="0" t="s">
-        <x:v>597</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="B128" s="0" t="s">
         <x:v>4</x:v>
@@ -8828,7 +9092,7 @@
     </x:row>
     <x:row r="129" spans="1:3">
       <x:c r="A129" s="0" t="s">
-        <x:v>598</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="B129" s="0" t="s">
         <x:v>4</x:v>
@@ -8839,7 +9103,7 @@
     </x:row>
     <x:row r="130" spans="1:3">
       <x:c r="A130" s="0" t="s">
-        <x:v>599</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="B130" s="0" t="s">
         <x:v>4</x:v>
@@ -8850,7 +9114,7 @@
     </x:row>
     <x:row r="131" spans="1:3">
       <x:c r="A131" s="0" t="s">
-        <x:v>600</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="B131" s="0" t="s">
         <x:v>4</x:v>
@@ -8861,7 +9125,7 @@
     </x:row>
     <x:row r="132" spans="1:3">
       <x:c r="A132" s="0" t="s">
-        <x:v>601</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="B132" s="0" t="s">
         <x:v>4</x:v>
@@ -8872,7 +9136,7 @@
     </x:row>
     <x:row r="133" spans="1:3">
       <x:c r="A133" s="0" t="s">
-        <x:v>602</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="B133" s="0" t="s">
         <x:v>4</x:v>
@@ -8883,7 +9147,7 @@
     </x:row>
     <x:row r="134" spans="1:3">
       <x:c r="A134" s="0" t="s">
-        <x:v>603</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="B134" s="0" t="s">
         <x:v>4</x:v>
@@ -8894,7 +9158,7 @@
     </x:row>
     <x:row r="135" spans="1:3">
       <x:c r="A135" s="0" t="s">
-        <x:v>604</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="B135" s="0" t="s">
         <x:v>4</x:v>
@@ -8905,7 +9169,7 @@
     </x:row>
     <x:row r="136" spans="1:3">
       <x:c r="A136" s="0" t="s">
-        <x:v>605</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="B136" s="0" t="s">
         <x:v>4</x:v>
@@ -8916,7 +9180,7 @@
     </x:row>
     <x:row r="137" spans="1:3">
       <x:c r="A137" s="0" t="s">
-        <x:v>606</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="B137" s="0" t="s">
         <x:v>4</x:v>
@@ -8927,276 +9191,12 @@
     </x:row>
     <x:row r="138" spans="1:3">
       <x:c r="A138" s="0" t="s">
-        <x:v>607</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="B138" s="0" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C138" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="139" spans="1:3">
-      <x:c r="A139" s="0" t="s">
-        <x:v>608</x:v>
-      </x:c>
-      <x:c r="B139" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C139" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="140" spans="1:3">
-      <x:c r="A140" s="0" t="s">
-        <x:v>609</x:v>
-      </x:c>
-      <x:c r="B140" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C140" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="141" spans="1:3">
-      <x:c r="A141" s="0" t="s">
-        <x:v>610</x:v>
-      </x:c>
-      <x:c r="B141" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C141" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="142" spans="1:3">
-      <x:c r="A142" s="0" t="s">
-        <x:v>611</x:v>
-      </x:c>
-      <x:c r="B142" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C142" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="143" spans="1:3">
-      <x:c r="A143" s="0" t="s">
-        <x:v>612</x:v>
-      </x:c>
-      <x:c r="B143" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C143" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="144" spans="1:3">
-      <x:c r="A144" s="0" t="s">
-        <x:v>613</x:v>
-      </x:c>
-      <x:c r="B144" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C144" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="145" spans="1:3">
-      <x:c r="A145" s="0" t="s">
-        <x:v>614</x:v>
-      </x:c>
-      <x:c r="B145" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C145" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="146" spans="1:3">
-      <x:c r="A146" s="0" t="s">
-        <x:v>615</x:v>
-      </x:c>
-      <x:c r="B146" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C146" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="147" spans="1:3">
-      <x:c r="A147" s="0" t="s">
-        <x:v>616</x:v>
-      </x:c>
-      <x:c r="B147" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C147" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="148" spans="1:3">
-      <x:c r="A148" s="0" t="s">
-        <x:v>617</x:v>
-      </x:c>
-      <x:c r="B148" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C148" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="149" spans="1:3">
-      <x:c r="A149" s="0" t="s">
-        <x:v>618</x:v>
-      </x:c>
-      <x:c r="B149" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C149" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="150" spans="1:3">
-      <x:c r="A150" s="0" t="s">
-        <x:v>619</x:v>
-      </x:c>
-      <x:c r="B150" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C150" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="151" spans="1:3">
-      <x:c r="A151" s="0" t="s">
-        <x:v>620</x:v>
-      </x:c>
-      <x:c r="B151" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C151" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="152" spans="1:3">
-      <x:c r="A152" s="0" t="s">
-        <x:v>621</x:v>
-      </x:c>
-      <x:c r="B152" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C152" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="153" spans="1:3">
-      <x:c r="A153" s="0" t="s">
-        <x:v>622</x:v>
-      </x:c>
-      <x:c r="B153" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C153" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="154" spans="1:3">
-      <x:c r="A154" s="0" t="s">
-        <x:v>623</x:v>
-      </x:c>
-      <x:c r="B154" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C154" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="155" spans="1:3">
-      <x:c r="A155" s="0" t="s">
-        <x:v>624</x:v>
-      </x:c>
-      <x:c r="B155" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C155" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="156" spans="1:3">
-      <x:c r="A156" s="0" t="s">
-        <x:v>625</x:v>
-      </x:c>
-      <x:c r="B156" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C156" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="157" spans="1:3">
-      <x:c r="A157" s="0" t="s">
-        <x:v>626</x:v>
-      </x:c>
-      <x:c r="B157" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C157" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="158" spans="1:3">
-      <x:c r="A158" s="0" t="s">
-        <x:v>627</x:v>
-      </x:c>
-      <x:c r="B158" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C158" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="159" spans="1:3">
-      <x:c r="A159" s="0" t="s">
-        <x:v>628</x:v>
-      </x:c>
-      <x:c r="B159" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C159" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="160" spans="1:3">
-      <x:c r="A160" s="0" t="s">
-        <x:v>629</x:v>
-      </x:c>
-      <x:c r="B160" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C160" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="161" spans="1:3">
-      <x:c r="A161" s="0" t="s">
-        <x:v>630</x:v>
-      </x:c>
-      <x:c r="B161" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C161" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="162" spans="1:3">
-      <x:c r="A162" s="0" t="s">
-        <x:v>631</x:v>
-      </x:c>
-      <x:c r="B162" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C162" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
     </x:row>

</xml_diff>